<commit_message>
update wordalisation for FAMD
</commit_message>
<xml_diff>
--- a/data/describe/few_shot/cluster/few_shot_cluster_description.xlsx
+++ b/data/describe/few_shot/cluster/few_shot_cluster_description.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2026FD1-B8F7-46A5-A467-72645216DC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4173E5B7-00E5-4A52-BB85-29225AE932BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{75A2F0CC-120C-46DD-B882-D3F79246B1DD}"/>
+    <workbookView xWindow="29940" yWindow="1140" windowWidth="22425" windowHeight="15225" xr2:uid="{75A2F0CC-120C-46DD-B882-D3F79246B1DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,28 +45,28 @@
     <t>Assistant</t>
   </si>
   <si>
-    <t>This cluster comprises highly creative individuals who are very engaged participants, while maintaining a normal level of confidence in their planning.
+    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical person in that cluster: ```Members of this cluster can be described as:  normal on confident planner,  relatively high on engaged participant,  quite high on creative´´´</t>
+  </si>
+  <si>
+    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical person in that cluster: ```Members of this cluster can be described as:  normal on principled,  normal on modern anxious,  very high on independent critical´´´</t>
+  </si>
+  <si>
+    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical dog in that cluster: ```Members of this cluster can be described as:  relatively high on calm and stable,  quite low on active and playful,  slightly low on self-reliant and composed,  normal on social and natural´´´</t>
+  </si>
+  <si>
+    <t>These individuals are highly creative and very engaged participants, while maintaining a normal level of confidence in their planning.
 Their significant creativity allows them to generate original ideas with ease, and their high engagement means they actively participate and confidently steer their own lives and emotions.
 Despite their strengths, their profound creativity can sometimes lead to feeling overwhelmed by their unique insights, and their self-directed approach may result in less spontaneous emotional connection with others.</t>
   </si>
   <si>
-    <t>This cluster is largely characterized by a profound skepticism towards established institutions, maintaining an average stance on both moral principles and modern anxieties.
+    <t>These individuals are largely characterized by a profound skepticism towards established institutions, maintaining an average stance on both moral principles and modern anxieties.
 Their strength lies in their highly independent and critical viewpoint, which fosters a diligent scrutiny of government, parliament, and political parties, potentially leading to greater accountability and an emphasis on personal agency.
 A potential weakness of this cluster is the very high level of distrust in vital civic structures, which could impede collective action or faith in the overall system.</t>
   </si>
   <si>
-    <t>This cluster describes dogs that are generally calm and stable, with low levels of activity and playfulness, and are slightly less self-reliant, while being average in their social tendencies.
+    <t>These  dogs that are generally calm and stable, with low levels of activity and playfulness, and are slightly less self-reliant, while being average in their social tendencies.
 Their primary strength lies in their calm and stable demeanor, meaning they don't demand extensive mental stimulation or high-energy activities.
 However, they are less inclined towards active play and might be less adaptable to new situations, and they may also exhibit less composure or independence when interacting with other dogs.</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical person in that cluster: ```Members of this cluster can be described as:  normal on confident planner,  relatively high on engaged participant,  quite high on creative´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical person in that cluster: ```Members of this cluster can be described as:  normal on principled,  normal on modern anxious,  very high on independent critical´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical dog in that cluster: ```Members of this cluster can be described as:  relatively high on calm and stable,  quite low on active and playful,  slightly low on self-reliant and composed,  normal on social and natural´´´</t>
   </si>
 </sst>
 </file>
@@ -446,26 +446,26 @@
     </row>
     <row r="2" spans="1:2" ht="134" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="137.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>